<commit_message>
Replace all em dashes with hyphens across entire project
Includes source code, comments, HTML, CSS, JS, Python generators,
Excel templates (regenerated), README, and CONTEXT docs.
Registry chartRows updated to match new Excel cell labels.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/Trial_2_v2_AI_SaaS.xlsx
+++ b/dashboard/Trial_2_v2_AI_SaaS.xlsx
@@ -750,7 +750,7 @@
       <c r="A2" s="44" t="n"/>
       <c r="B2" s="45" t="inlineStr">
         <is>
-          <t>THE VC CORNER — Quick Start Guide</t>
+          <t>THE VC CORNER - Quick Start Guide</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       <c r="A12" s="44" t="n"/>
       <c r="B12" s="46" t="inlineStr">
         <is>
-          <t>Open the sheet matching your Business Type (AI-SaaS, D2C, or Healthcare). Fill only the blue cells — these are your inputs. Gray cells with formulas will auto-calculate. Enter 5-year projections in columns B through F.</t>
+          <t>Open the sheet matching your Business Type (AI-SaaS, D2C, or Healthcare). Fill only the blue cells - these are your inputs. Gray cells with formulas will auto-calculate. Enter 5-year projections in columns B through F.</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       <c r="A15" s="44" t="n"/>
       <c r="B15" s="46" t="inlineStr">
         <is>
-          <t>Save this file, then go to thevcorner.com. Click 'Upload Template' and select your saved .xlsx file. Everything runs in your browser — your data never leaves your device.</t>
+          <t>Save this file, then go to thevcorner.com. Click 'Upload Template' and select your saved .xlsx file. Everything runs in your browser - your data never leaves your device.</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="C22" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Your input — fill these cells</t>
+          <t xml:space="preserve">  Your input - fill these cells</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="C23" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Auto-calculated (formula) — do not edit</t>
+          <t xml:space="preserve">  Auto-calculated (formula) - do not edit</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       <c r="A27" s="44" t="n"/>
       <c r="B27" s="53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •  Only fill sections you marked 'Yes' on the Checklist — everything else is ignored.</t>
+          <t xml:space="preserve">  •  Only fill sections you marked 'Yes' on the Checklist - everything else is ignored.</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       <c r="A30" s="44" t="n"/>
       <c r="B30" s="53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  •  Upload your completed file at thevcorner.com — 100% private, browser-only processing.</t>
+          <t xml:space="preserve">  •  Upload your completed file at thevcorner.com - 100% private, browser-only processing.</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — Company Setup</t>
+          <t>THE VC CORNER - Company Setup</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — Section Checklist</t>
+          <t>THE VC CORNER - Section Checklist</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
 • Set each section to Yes or No
 • Only 'Yes' sections appear on the dashboard
 • The original 10 sections per sector default to Yes
-• New v2 sections default to No — enable as needed</t>
+• New v2 sections default to No - enable as needed</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — AI-SaaS Projections</t>
+          <t>THE VC CORNER - AI-SaaS Projections</t>
         </is>
       </c>
     </row>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="D82" s="38" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E82" s="38" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="F82" s="38" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -6471,7 +6471,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — D2C Projections</t>
+          <t>THE VC CORNER - D2C Projections</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6597,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GMV — Website</t>
+          <t xml:space="preserve">  GMV - Website</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -6692,7 +6692,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GMV — Retail</t>
+          <t xml:space="preserve">  GMV - Retail</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -6787,7 +6787,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GMV — Marketplace</t>
+          <t xml:space="preserve">  GMV - Marketplace</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -6889,7 +6889,7 @@
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>Website — GMV</t>
+          <t>Website - GMV</t>
         </is>
       </c>
       <c r="B24" s="18" t="n"/>
@@ -6906,7 +6906,7 @@
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>Website — Return Rate</t>
+          <t>Website - Return Rate</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -6923,7 +6923,7 @@
     <row r="26">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>Website — Net Revenue</t>
+          <t>Website - Net Revenue</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -6955,7 +6955,7 @@
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>Retail — GMV</t>
+          <t>Retail - GMV</t>
         </is>
       </c>
       <c r="B27" s="18" t="n"/>
@@ -6972,7 +6972,7 @@
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
         <is>
-          <t>Retail — Return Rate</t>
+          <t>Retail - Return Rate</t>
         </is>
       </c>
       <c r="B28" s="27" t="n"/>
@@ -6989,7 +6989,7 @@
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>Retail — Net Revenue</t>
+          <t>Retail - Net Revenue</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -7021,7 +7021,7 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — GMV</t>
+          <t>Marketplace - GMV</t>
         </is>
       </c>
       <c r="B30" s="18" t="n"/>
@@ -7038,7 +7038,7 @@
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Return Rate</t>
+          <t>Marketplace - Return Rate</t>
         </is>
       </c>
       <c r="B31" s="27" t="n"/>
@@ -7055,7 +7055,7 @@
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Commission %</t>
+          <t>Marketplace - Commission %</t>
         </is>
       </c>
       <c r="B32" s="27" t="n"/>
@@ -7072,7 +7072,7 @@
     <row r="33">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>Marketplace — Net Revenue</t>
+          <t>Marketplace - Net Revenue</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -7157,7 +7157,7 @@
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>Website — Gross Revenue</t>
+          <t>Website - Gross Revenue</t>
         </is>
       </c>
       <c r="B37" s="18" t="n"/>
@@ -7174,7 +7174,7 @@
     <row r="38">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>Website — Returns</t>
+          <t>Website - Returns</t>
         </is>
       </c>
       <c r="B38" s="18" t="n"/>
@@ -7191,7 +7191,7 @@
     <row r="39">
       <c r="A39" s="19" t="inlineStr">
         <is>
-          <t>Website — Net Revenue</t>
+          <t>Website - Net Revenue</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -7223,7 +7223,7 @@
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>Retail — Gross Revenue</t>
+          <t>Retail - Gross Revenue</t>
         </is>
       </c>
       <c r="B40" s="18" t="n"/>
@@ -7240,7 +7240,7 @@
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>Retail — Returns</t>
+          <t>Retail - Returns</t>
         </is>
       </c>
       <c r="B41" s="18" t="n"/>
@@ -7257,7 +7257,7 @@
     <row r="42">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>Retail — Net Revenue</t>
+          <t>Retail - Net Revenue</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -7289,7 +7289,7 @@
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Gross Revenue</t>
+          <t>Marketplace - Gross Revenue</t>
         </is>
       </c>
       <c r="B43" s="18" t="n"/>
@@ -7306,7 +7306,7 @@
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Returns</t>
+          <t>Marketplace - Returns</t>
         </is>
       </c>
       <c r="B44" s="18" t="n"/>
@@ -7323,7 +7323,7 @@
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Commission</t>
+          <t>Marketplace - Commission</t>
         </is>
       </c>
       <c r="B45" s="18" t="n"/>
@@ -7340,7 +7340,7 @@
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
         <is>
-          <t>Marketplace — Net Revenue</t>
+          <t>Marketplace - Net Revenue</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -7546,7 +7546,7 @@
     <row r="57">
       <c r="A57" s="17" t="inlineStr">
         <is>
-          <t>Website — Churn Rate</t>
+          <t>Website - Churn Rate</t>
         </is>
       </c>
       <c r="B57" s="27" t="n"/>
@@ -7563,7 +7563,7 @@
     <row r="58">
       <c r="A58" s="17" t="inlineStr">
         <is>
-          <t>Retail — Churn Rate</t>
+          <t>Retail - Churn Rate</t>
         </is>
       </c>
       <c r="B58" s="27" t="n"/>
@@ -7580,7 +7580,7 @@
     <row r="59">
       <c r="A59" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Churn Rate</t>
+          <t>Marketplace - Churn Rate</t>
         </is>
       </c>
       <c r="B59" s="27" t="n"/>
@@ -9806,7 +9806,7 @@
     <row r="181">
       <c r="A181" s="17" t="inlineStr">
         <is>
-          <t>Website — Revenue</t>
+          <t>Website - Revenue</t>
         </is>
       </c>
       <c r="B181" s="18" t="n"/>
@@ -9823,7 +9823,7 @@
     <row r="182">
       <c r="A182" s="17" t="inlineStr">
         <is>
-          <t>Website — Variable Cost</t>
+          <t>Website - Variable Cost</t>
         </is>
       </c>
       <c r="B182" s="18" t="n"/>
@@ -9840,7 +9840,7 @@
     <row r="183">
       <c r="A183" s="19" t="inlineStr">
         <is>
-          <t>Website — Contribution Margin</t>
+          <t>Website - Contribution Margin</t>
         </is>
       </c>
       <c r="B183" s="20">
@@ -9872,7 +9872,7 @@
     <row r="184">
       <c r="A184" s="17" t="inlineStr">
         <is>
-          <t>Retail — Revenue</t>
+          <t>Retail - Revenue</t>
         </is>
       </c>
       <c r="B184" s="18" t="n"/>
@@ -9889,7 +9889,7 @@
     <row r="185">
       <c r="A185" s="17" t="inlineStr">
         <is>
-          <t>Retail — Variable Cost</t>
+          <t>Retail - Variable Cost</t>
         </is>
       </c>
       <c r="B185" s="18" t="n"/>
@@ -9906,7 +9906,7 @@
     <row r="186">
       <c r="A186" s="19" t="inlineStr">
         <is>
-          <t>Retail — Contribution Margin</t>
+          <t>Retail - Contribution Margin</t>
         </is>
       </c>
       <c r="B186" s="20">
@@ -9938,7 +9938,7 @@
     <row r="187">
       <c r="A187" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Revenue</t>
+          <t>Marketplace - Revenue</t>
         </is>
       </c>
       <c r="B187" s="18" t="n"/>
@@ -9955,7 +9955,7 @@
     <row r="188">
       <c r="A188" s="17" t="inlineStr">
         <is>
-          <t>Marketplace — Variable Cost</t>
+          <t>Marketplace - Variable Cost</t>
         </is>
       </c>
       <c r="B188" s="18" t="n"/>
@@ -9972,7 +9972,7 @@
     <row r="189">
       <c r="A189" s="19" t="inlineStr">
         <is>
-          <t>Marketplace — Contribution Margin</t>
+          <t>Marketplace - Contribution Margin</t>
         </is>
       </c>
       <c r="B189" s="20">
@@ -10419,7 +10419,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE VC CORNER — Healthcare Projections</t>
+          <t>THE VC CORNER - Healthcare Projections</t>
         </is>
       </c>
     </row>

</xml_diff>